<commit_message>
Update QA test case documentation
- Add bug reports for signup password limit and missing subreplies

- Add session hijacking test evidence PDF

- Update authentication test case workbooks and bug report template

- Remove duplicate completed login workbook
</commit_message>
<xml_diff>
--- a/qa-docs/test-cases/Done/Authentication/VerseByVerse_Authorization_Test_Cases.xlsx
+++ b/qa-docs/test-cases/Done/Authentication/VerseByVerse_Authorization_Test_Cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\versebyverse-quality-engineering\qa-docs\test-cases\Authentication\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\versebyverse-quality-engineering\qa-docs\test-cases\Done\Authentication\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B50B62C-F9DA-47C8-80C2-9C326103F9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CBFD771-A565-4D99-A597-30D2758BA558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Authorization Test Cases" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="100">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -116,9 +116,6 @@
     <t>No active session</t>
   </si>
   <si>
-    <t>1. Send request to protected API endpoint</t>
-  </si>
-  <si>
     <t>API returns 401 Unauthorized
 No data is returned</t>
   </si>
@@ -304,9 +301,6 @@
   <si>
     <t>API rejects request
 Proper authorization enforced</t>
-  </si>
-  <si>
-    <t>Fail</t>
   </si>
   <si>
     <t>1. Navigate directly to protected route URL
@@ -318,6 +312,49 @@
     <t xml:space="preserve">Access is denied
 User is redirected to the protected route's root walkthrough page
 For profile page, user is redirected to the login page
+</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Logged-out protected routes now redirect by feature area instead of always going to sign-in.</t>
+  </si>
+  <si>
+    <t>User is directed to the respected walkthrough or signin page</t>
+  </si>
+  <si>
+    <t>Access is denied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API returns 401 Unauthorized
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API returns success response with meta data
+</t>
+  </si>
+  <si>
+    <t>1. Send request to protected API endpoint
+eg. 
+fetch("/community/my", { credentials: "include" })
+  .then(async (res) =&gt; ({ status: res.status, body: await res.text() }))
+  .then(console.log);</t>
+  </si>
+  <si>
+    <t>Fixed - Leader / Ownder only actions are entirely disabled from member view</t>
+  </si>
+  <si>
+    <t>Access is denied
+*fix - User is logged out</t>
+  </si>
+  <si>
+    <t>Request is Rejected
+401, Not authenticated thrown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access is denied
+User is signed out and requested to sign in again
 </t>
   </si>
 </sst>
@@ -359,13 +396,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -679,7 +719,7 @@
     <col min="5" max="5" width="25" customWidth="1"/>
     <col min="6" max="6" width="50" customWidth="1"/>
     <col min="7" max="7" width="40" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="8" max="8" width="32.42578125" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
     <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
@@ -733,18 +773,20 @@
         <v>14</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -766,11 +808,15 @@
       <c r="G3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
@@ -792,11 +838,15 @@
       <c r="G4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>26</v>
       </c>
@@ -813,21 +863,25 @@
         <v>29</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="J5" s="2"/>
+    </row>
+    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>17</v>
@@ -836,276 +890,320 @@
         <v>28</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J6" s="2"/>
     </row>
     <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="J7" s="2"/>
+    </row>
+    <row r="8" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J8" s="2"/>
     </row>
     <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="H9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J9" s="2"/>
     </row>
     <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J10" s="2"/>
     </row>
     <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="H11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J11" s="2"/>
     </row>
     <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E13" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
+      <c r="H13" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>75</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="G14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+      <c r="H14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="G15" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+      <c r="H15" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J15" s="2"/>
     </row>
     <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F16" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
+      <c r="H16" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="J16" s="2"/>
     </row>
   </sheetData>

</xml_diff>